<commit_message>
Lista de compras agrupada pelo grupo do alimento
dominio/gruposDaLista (agruparLista: grupos em ordem alfabética sem
acento, "Outros itens" e "Adicionados por você" no fim; sugerirGrupos)
com testes. A linha da lista leva o grupo do item publicado; a prévia do
treinador recebe o grupo atual por /alimentos/fatores. Tela do aluno,
prévia e PDFs (lista e Detalhado da dieta) em grupos com a contagem, sem
mudar a conta nem o "N de M comprados". Campo Grupo com sugestões em
Biblioteca › Alimentos, coluna Grupo na importação (modelos regerados),
Ajuda e e2e da lista de compras.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DrMBZ6rsocVMngqf7kS5sS
</commit_message>
<xml_diff>
--- a/app/public/modelos/importacao/alimentos.xlsx
+++ b/app/public/modelos/importacao/alimentos.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -44,6 +44,9 @@
     <t xml:space="preserve">FCc</t>
   </si>
   <si>
+    <t xml:space="preserve">Grupo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aveia fictícia</t>
   </si>
   <si>
@@ -71,6 +74,9 @@
     <t xml:space="preserve">Tabela fictícia</t>
   </si>
   <si>
+    <t xml:space="preserve">Cereais e derivados</t>
+  </si>
+  <si>
     <t xml:space="preserve">Iogurte fictício</t>
   </si>
   <si>
@@ -86,6 +92,9 @@
     <t xml:space="preserve">3</t>
   </si>
   <si>
+    <t xml:space="preserve">Leite e derivados</t>
+  </si>
+  <si>
     <t xml:space="preserve">Suco fictício</t>
   </si>
   <si>
@@ -159,6 +168,9 @@
   </si>
   <si>
     <t xml:space="preserve">2,5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 60 letras. Agrupa a lista de compras do aluno. Vazio fica em "Outros itens".</t>
   </si>
   <si>
     <t xml:space="preserve">A primeira linha da aba Dados é o cabeçalho.</t>
@@ -221,110 +233,122 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K2" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="L2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K3" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="L3" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K4" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="L4" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -336,16 +360,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2">
@@ -353,13 +377,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -367,13 +391,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -381,27 +405,27 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
         <v>41</v>
       </c>
-      <c r="B5" t="s">
-        <v>38</v>
-      </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -409,13 +433,13 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -423,13 +447,13 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -437,13 +461,13 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -451,111 +475,125 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>